<commit_message>
Added excel reader for test case 4
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497745_cognizant_com/Documents/Documents/HackathonProject/InsuranceAutomationHackathon/src/test/java/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497788\IdeaProjects\HackathonProject\InsuranceAutomationHackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="11_F25DC773A252ABDACC104848599D7EA05BDE58FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC801BE-855C-4417-94E3-A354BC8867E2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03907A8E-82F2-40F6-B540-F741D4B22753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Car" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="79">
   <si>
     <t>CityOfRegistration</t>
   </si>
@@ -237,13 +237,40 @@
   </si>
   <si>
     <t>KARNATAKA-BANGALORE</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>Email ID</t>
+  </si>
+  <si>
+    <t>Mobile Number</t>
+  </si>
+  <si>
+    <t>PinCode</t>
+  </si>
+  <si>
+    <t>John Wick</t>
+  </si>
+  <si>
+    <t>Amy</t>
+  </si>
+  <si>
+    <t>xyz@abc.com</t>
+  </si>
+  <si>
+    <t>man@abc.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +295,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -305,10 +340,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -320,8 +356,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -335,10 +381,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -953,9 +995,72 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFF976E0-C036-4A05-969A-5FBEA2A39948}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21.81640625" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" customWidth="1"/>
+    <col min="3" max="3" width="20.26953125" customWidth="1"/>
+    <col min="4" max="4" width="16.90625" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="6">
+        <v>9876123450</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="6">
+        <v>628503</v>
+      </c>
+      <c r="E2" s="5">
+        <v>17394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="6">
+        <v>9876321450</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="6">
+        <v>625011</v>
+      </c>
+      <c r="E3" s="5">
+        <v>37987</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{E647BBDA-5D91-4146-A026-E3E7E59B8288}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{CA018CC8-BC8A-43F1-A7DD-07604930BDF9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
testcase 21-25 are converted to standalone
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hackathon Projects\InsuranceAutomationHackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65C7259-9217-422A-8DB8-FD77DA36F335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E2AB5E-44B5-40C5-8B5B-C993112DA8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -315,7 +315,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -336,11 +336,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="7" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -980,63 +983,66 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.26953125" customWidth="1"/>
+    <col min="4" max="4" width="10.08984375" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="H1" s="7"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="9">
         <v>37084</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="8">
         <v>9876543210</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="7">
+      <c r="G2" s="8">
         <v>628008</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>68</v>
-      </c>
+      <c r="H2" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{F53E2C14-C1B6-49C1-AEAB-A5CEF0E710EA}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{F53E2C14-C1B6-49C1-AEAB-A5CEF0E710EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
testcase 21-24 are converted to standalone
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hackathon Projects\InsuranceAutomationHackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E2AB5E-44B5-40C5-8B5B-C993112DA8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67CA3B1-33B7-44F7-9FDC-C6AC358E8768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="71">
   <si>
     <t>CityOfRegistration</t>
   </si>
@@ -229,6 +229,12 @@
   </si>
   <si>
     <t>Amy</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Activate Booster</t>
   </si>
 </sst>
 </file>
@@ -983,9 +989,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
     <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.08984375" customWidth="1"/>
     <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -1040,9 +1047,33 @@
       </c>
       <c r="H2" s="7"/>
     </row>
+    <row r="3" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="9">
+        <v>37085</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="8">
+        <v>9876543211</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="8">
+        <v>620018</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{F53E2C14-C1B6-49C1-AEAB-A5CEF0E710EA}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{222AE723-77D7-4EDE-8AF6-7993B87FD074}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
Final TravelPages and Testcases update
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hackathon Projects\InsuranceAutomationHackathon\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497728_cognizant_com/Documents/Documents/LombardProject/PolicyBazzarAutomationHackathon/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67CA3B1-33B7-44F7-9FDC-C6AC358E8768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{A67CA3B1-33B7-44F7-9FDC-C6AC358E8768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA02E141-D5A7-422D-9367-15653EDEF475}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Car" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="64">
   <si>
     <t>CityOfRegistration</t>
   </si>
@@ -114,12 +114,6 @@
     <t>Germany</t>
   </si>
   <si>
-    <t>12, Oct 2026</t>
-  </si>
-  <si>
-    <t>25, Oct 2026</t>
-  </si>
-  <si>
     <t>Italy</t>
   </si>
   <si>
@@ -129,15 +123,6 @@
     <t>30, Sept 2026</t>
   </si>
   <si>
-    <t>Spain</t>
-  </si>
-  <si>
-    <t>21, Aug 2026</t>
-  </si>
-  <si>
-    <t>27, Nov 2026</t>
-  </si>
-  <si>
     <t>22,21</t>
   </si>
   <si>
@@ -159,18 +144,12 @@
     <t>SeniorTravelDOB</t>
   </si>
   <si>
-    <t>77,29,34</t>
-  </si>
-  <si>
     <t>81,58,33,76</t>
   </si>
   <si>
     <t>81=16-08-1944,76=17-07-1949</t>
   </si>
   <si>
-    <t>77=09-06-1948</t>
-  </si>
-  <si>
     <t>81,33,76</t>
   </si>
   <si>
@@ -186,9 +165,6 @@
     <t>28, Oct 2026</t>
   </si>
   <si>
-    <t>Ukraine</t>
-  </si>
-  <si>
     <t>24, Dec 2026</t>
   </si>
   <si>
@@ -235,6 +211,9 @@
   </si>
   <si>
     <t>Activate Booster</t>
+  </si>
+  <si>
+    <t>Portugal</t>
   </si>
 </sst>
 </file>
@@ -321,7 +300,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -336,9 +315,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -775,7 +751,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA02EFBC-3215-45E3-811B-5BCF5E5AE3DE}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -805,13 +781,13 @@
         <v>25</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -828,32 +804,32 @@
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D3" s="3">
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H3">
         <v>54</v>
@@ -861,124 +837,77 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="3">
-        <v>1</v>
-      </c>
-      <c r="E4" s="3">
-        <v>45</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="G4" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H4">
-        <v>45</v>
+        <v>36</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="3">
-        <v>3</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="3">
-        <v>4</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1000,73 +929,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C2" s="8">
+        <v>37084</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="7">
+        <v>9876543210</v>
+      </c>
+      <c r="F2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" s="8" t="s">
+      <c r="G2" s="7">
+        <v>628008</v>
+      </c>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="8">
+        <v>37085</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="7"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="9">
-        <v>37084</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="8">
-        <v>9876543210</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="G2" s="8">
-        <v>628008</v>
-      </c>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="9">
-        <v>37085</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <v>9876543211</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="G3" s="8">
+      <c r="F3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="7">
         <v>620018</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finallized TravelPages and Testcases update
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497728_cognizant_com/Documents/Documents/LombardProject/PolicyBazzarAutomationHackathon/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{A67CA3B1-33B7-44F7-9FDC-C6AC358E8768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEE31A6F-E120-4D41-A1C7-0069C6B0D967}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{A67CA3B1-33B7-44F7-9FDC-C6AC358E8768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A3E6AED-31A6-43A8-A9F1-8A995AAA93F0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
   <si>
     <t>CityOfRegistration</t>
   </si>
@@ -138,21 +138,9 @@
     <t>HealthIssueTravellers</t>
   </si>
   <si>
-    <t>22,33,76</t>
-  </si>
-  <si>
     <t>SeniorTravelDOB</t>
   </si>
   <si>
-    <t>81,58,33,76</t>
-  </si>
-  <si>
-    <t>81=16-08-1944,76=17-07-1949</t>
-  </si>
-  <si>
-    <t>81,33,76</t>
-  </si>
-  <si>
     <t>UK</t>
   </si>
   <si>
@@ -168,9 +156,6 @@
     <t>1, Jan 2027</t>
   </si>
   <si>
-    <t>54,7,21</t>
-  </si>
-  <si>
     <t>Product</t>
   </si>
   <si>
@@ -219,10 +204,28 @@
     <t>21, Nov 2026</t>
   </si>
   <si>
-    <t>81,58</t>
-  </si>
-  <si>
-    <t>85=16-08-1941</t>
+    <t>85=26-09-1941</t>
+  </si>
+  <si>
+    <t>72,58,33</t>
+  </si>
+  <si>
+    <t>81,33,77,52</t>
+  </si>
+  <si>
+    <t>72=21-12-1954</t>
+  </si>
+  <si>
+    <t>22,33,77</t>
+  </si>
+  <si>
+    <t>85,58</t>
+  </si>
+  <si>
+    <t>54,7,37</t>
+  </si>
+  <si>
+    <t>81=16-08-1944,77=09-11-1948</t>
   </si>
 </sst>
 </file>
@@ -794,7 +797,7 @@
         <v>25</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>34</v>
@@ -829,16 +832,16 @@
         <v>29</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D3" s="3">
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="4" t="s">
@@ -859,56 +862,56 @@
         <v>32</v>
       </c>
       <c r="D4" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="3">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>42</v>
+      <c r="H5" s="4">
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>
@@ -917,7 +920,7 @@
         <v>65</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>35</v>
@@ -943,46 +946,46 @@
   <sheetData>
     <row r="1" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C2" s="8">
         <v>37084</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E2" s="7">
         <v>9876543210</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G2" s="7">
         <v>628008</v>
@@ -991,22 +994,22 @@
     </row>
     <row r="3" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C3" s="8">
         <v>37085</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E3" s="7">
         <v>9876543211</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G3" s="7">
         <v>620018</v>

</xml_diff>